<commit_message>
Update for January 17, 2025
</commit_message>
<xml_diff>
--- a/python/data/Revenue_Report.xlsx
+++ b/python/data/Revenue_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,163 +427,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-01-12T16:00:00.000Z</v>
+        <v>2026-01-17</v>
       </c>
       <c r="B2" t="str">
-        <v>Gretchen B. Olivar</v>
+        <v>MERLYN LEOCADIO ANAJAO</v>
       </c>
       <c r="C2" t="str">
         <v>Sigfred Navasquez</v>
       </c>
       <c r="D2" t="str">
-        <v>Extraction - 3</v>
+        <v>Oral Prophylaxis - 32</v>
       </c>
       <c r="E2" t="str">
         <v>Basic Procedure</v>
       </c>
       <c r="F2" t="str">
-        <v>2400.00</v>
+        <v>1000.00</v>
       </c>
       <c r="G2" t="str">
-        <v>1440.00</v>
+        <v>600.00</v>
       </c>
       <c r="H2" t="str">
-        <v>960.00</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2026-02-01T16:00:00.000Z</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Gretchen B. Olivar</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Sigfred Navasquez</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Brace - 16</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Special Case</v>
-      </c>
-      <c r="F3" t="str">
-        <v>12800.00</v>
-      </c>
-      <c r="G3" t="str">
-        <v>6400.00</v>
-      </c>
-      <c r="H3" t="str">
-        <v>6400.00</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2026-02-02T16:00:00.000Z</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Gretchen B. Olivar</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sigfred Navasquez</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Brace - 16</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Special Case</v>
-      </c>
-      <c r="F4" t="str">
-        <v>12800.00</v>
-      </c>
-      <c r="G4" t="str">
-        <v>6400.00</v>
-      </c>
-      <c r="H4" t="str">
-        <v>6400.00</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-03-08T16:00:00.000Z</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Gretchen B. Olivar</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Sigfred Navasquez</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Extraction - 32</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Basic Procedure</v>
-      </c>
-      <c r="F5" t="str">
-        <v>25600.00</v>
-      </c>
-      <c r="G5" t="str">
-        <v>15360.00</v>
-      </c>
-      <c r="H5" t="str">
-        <v>10240.00</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2026-03-09T16:00:00.000Z</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Gretchen B. Olivar</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Sigfred Navasquez</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Brace - 16</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Special Case</v>
-      </c>
-      <c r="F6" t="str">
-        <v>12800.00</v>
-      </c>
-      <c r="G6" t="str">
-        <v>6400.00</v>
-      </c>
-      <c r="H6" t="str">
-        <v>6400.00</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>2026-01-09T16:00:00.000Z</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Gretchen B. Olivar</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Sigfred Navasquez</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Extraction - 4</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Basic Procedure</v>
-      </c>
-      <c r="F7" t="str">
-        <v>3200.00</v>
-      </c>
-      <c r="G7" t="str">
-        <v>1920.00</v>
-      </c>
-      <c r="H7" t="str">
-        <v>1280.00</v>
+        <v>400.00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>